<commit_message>
Lead extraction 2026-08-11 (weekly, slk)
</commit_message>
<xml_diff>
--- a/UT/slk/2026-08-11.xlsx
+++ b/UT/slk/2026-08-11.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -460,6 +460,69 @@
       <c r="I1" t="inlineStr">
         <is>
           <t>Obituary URL</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Posted Date</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Property Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Thomas Edwin "Ed" Barton</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>BARTON, THOMAS E; TR (TEB FAM LIV TRUST)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>22-33-251-011-0000</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>1749 E VISCOUNTI DR</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>SANDY</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>84093</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>initial E matches deceased's own name 'Edwin'</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>$ 681,400</t>
         </is>
       </c>
     </row>

</xml_diff>